<commit_message>
Update scenario matrix Excel output
</commit_message>
<xml_diff>
--- a/artifacts/generated/qa/scenario-matrix.xlsx
+++ b/artifacts/generated/qa/scenario-matrix.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Scenario Matrix" sheetId="1" r:id="rId1"/>
+    <sheet name="測試情境" sheetId="1" r:id="rId1"/>
+    <sheet name="測試案例" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -167,7 +168,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -183,7 +184,7 @@
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="62" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -209,7 +210,7 @@
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t>狀態</t>
+          <t>情境狀態</t>
         </is>
       </c>
     </row>
@@ -233,12 +234,12 @@
       </c>
       <c r="C3" t="inlineStr" s="12">
         <is>
-          <t>點擊「忘記密碼」 -&gt; 進入忘記密碼流程。</t>
+          <t>給定使用者位於登入頁，當點擊「忘記密碼」 -&gt; 進入忘記密碼流程</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="13">
@@ -260,12 +261,12 @@
       </c>
       <c r="C4" t="inlineStr" s="12">
         <is>
-          <t>未輸入 Email 就送出 -&gt; 提示 Email 為必填。</t>
+          <t>給定使用者位於忘記密碼頁，當未輸入 Email 就送出 -&gt; 提示 Email 為必填</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="13">
@@ -287,12 +288,12 @@
       </c>
       <c r="C5" t="inlineStr" s="12">
         <is>
-          <t>輸入格式錯誤的 Email 並送出 -&gt; 提示 Email 格式錯誤。</t>
+          <t>給定使用者位於忘記密碼頁，當輸入格式錯誤的 Email 並送出 -&gt; 提示 Email 格式錯誤</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="13">
@@ -314,12 +315,12 @@
       </c>
       <c r="C6" t="inlineStr" s="12">
         <is>
-          <t>輸入有效 Email 並送出 -&gt; 提示已送出密碼重設通知。</t>
+          <t>給定使用者位於忘記密碼頁，當輸入有效 Email 並送出 -&gt; 提示已送出密碼重設通知</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="13">
@@ -341,12 +342,12 @@
       </c>
       <c r="C7" t="inlineStr" s="12">
         <is>
-          <t>使用者輸入有效帳號與正確密碼並送出 -&gt; 登入成功。</t>
+          <t>給定使用者位於登入頁，當使用者輸入有效帳號與正確密碼並送出 -&gt; 登入成功</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="13">
@@ -368,12 +369,12 @@
       </c>
       <c r="C8" t="inlineStr" s="12">
         <is>
-          <t>使用者未輸入帳號就送出 -&gt; 提示帳號為必填。</t>
+          <t>給定使用者位於登入頁，當使用者未輸入帳號就送出 -&gt; 提示帳號為必填</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="13">
@@ -395,12 +396,12 @@
       </c>
       <c r="C9" t="inlineStr" s="12">
         <is>
-          <t>使用者未輸入密碼就送出 -&gt; 提示密碼為必填。</t>
+          <t>給定使用者位於登入頁，當使用者未輸入密碼就送出 -&gt; 提示密碼為必填</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="13">
@@ -422,12 +423,12 @@
       </c>
       <c r="C10" t="inlineStr" s="12">
         <is>
-          <t>使用者輸入錯誤帳號或錯誤密碼並送出 -&gt; 顯示登入失敗提示。</t>
+          <t>給定使用者位於登入頁，當使用者輸入錯誤帳號或錯誤密碼並送出 -&gt; 顯示登入失敗提示</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="13">
@@ -449,12 +450,12 @@
       </c>
       <c r="C11" t="inlineStr" s="12">
         <is>
-          <t>使用者點擊「忘記密碼」 -&gt; 導向忘記密碼流程。</t>
+          <t>給定使用者位於登入頁，當使用者點擊「忘記密碼」 -&gt; 導向忘記密碼流程</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="13">
@@ -476,12 +477,12 @@
       </c>
       <c r="C12" t="inlineStr" s="12">
         <is>
-          <t>使用者點擊「創建帳號」 -&gt; 導向註冊流程。</t>
+          <t>給定使用者位於登入頁，當使用者點擊「創建帳號」 -&gt; 導向註冊流程</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="13">
@@ -503,12 +504,12 @@
       </c>
       <c r="C13" t="inlineStr" s="12">
         <is>
-          <t>點擊「創建帳號」 -&gt; 進入註冊流程。</t>
+          <t>給定使用者位於登入頁，當點擊「創建帳號」 -&gt; 進入註冊流程</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E13" t="inlineStr" s="13">
@@ -530,12 +531,12 @@
       </c>
       <c r="C14" t="inlineStr" s="12">
         <is>
-          <t>必填欄位未填就送出 -&gt; 提示必填欄位。</t>
+          <t>給定使用者位於註冊頁，當必填欄位未填就送出 -&gt; 提示必填欄位</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="13">
@@ -557,12 +558,12 @@
       </c>
       <c r="C15" t="inlineStr" s="12">
         <is>
-          <t>密碼與確認密碼不一致並送出 -&gt; 提示密碼不一致。</t>
+          <t>給定使用者位於註冊頁，當密碼與確認密碼不一致並送出 -&gt; 提示密碼不一致</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="13">
@@ -584,12 +585,12 @@
       </c>
       <c r="C16" t="inlineStr" s="12">
         <is>
-          <t>輸入有效資料並送出 -&gt; 建立帳號或進入後續驗證流程。</t>
+          <t>給定使用者位於註冊頁，當輸入有效資料並送出 -&gt; 建立帳號或進入後續驗證流程</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="11">
         <is>
-          <t>—</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="13">
@@ -608,5 +609,909 @@
     <mergeCell ref="A7:A12"/>
     <mergeCell ref="A13:A16"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D3:D16">
+      <formula1>"Not Run,Ready,Pass,Fail,Blocked,N/A"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E3:E16">
+      <formula1>"Not Marked,Ready,Need Confirm,Approved,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="9" width="38" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="42" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>功能模組</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>測試案例 ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>對應情境 ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>標題</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>類型</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t>優先級</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>前置條件</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t>步驟</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>預期結果</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t>自動化建議</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="82" customHeight="1">
+      <c r="A2" t="inlineStr" s="13">
+        <is>
+          <t>forgot-password</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="13">
+        <is>
+          <t>TC-FORGOT-PASSWORD-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="13">
+        <is>
+          <t>SC-FORGOT-PASSWORD-001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="12">
+        <is>
+          <t>忘記密碼入口導向正確</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於登入頁</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr" s="12">
+        <is>
+          <t>1. 點擊忘記密碼入口</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統進入忘記密碼流程</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr" s="12">
+        <is>
+          <t>導向 URL 或頁面狀態需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="82" customHeight="1">
+      <c r="A3" t="inlineStr" s="13">
+        <is>
+          <t>forgot-password</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="13">
+        <is>
+          <t>TC-FORGOT-PASSWORD-002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="13">
+        <is>
+          <t>SC-FORGOT-PASSWORD-002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="12">
+        <is>
+          <t>忘記密碼未輸入 Email 時提示必填</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於忘記密碼頁</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr" s="12">
+        <is>
+          <t>1. 保留 Email 欄位空白
+2. 送出申請</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統提示 Email 為必填</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr" s="12">
+        <is>
+          <t>提示文案需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="82" customHeight="1">
+      <c r="A4" t="inlineStr" s="13">
+        <is>
+          <t>forgot-password</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="13">
+        <is>
+          <t>TC-FORGOT-PASSWORD-003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="13">
+        <is>
+          <t>SC-FORGOT-PASSWORD-003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="12">
+        <is>
+          <t>忘記密碼輸入錯誤 Email 格式時提示錯誤</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於忘記密碼頁</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="12">
+        <is>
+          <t>1. 輸入格式錯誤的 Email
+2. 送出申請</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統提示 Email 格式錯誤</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr" s="12">
+        <is>
+          <t>錯誤格式樣本與文案需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="82" customHeight="1">
+      <c r="A5" t="inlineStr" s="13">
+        <is>
+          <t>forgot-password</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="13">
+        <is>
+          <t>TC-FORGOT-PASSWORD-004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="13">
+        <is>
+          <t>SC-FORGOT-PASSWORD-004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="12">
+        <is>
+          <t>忘記密碼輸入有效 Email 後送出通知</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於忘記密碼頁
+2. 測試 Email 可用</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr" s="12">
+        <is>
+          <t>1. 輸入有效 Email
+2. 送出申請</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統提示已送出密碼重設通知</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr" s="12">
+        <is>
+          <t>是否實際驗證信件送達需依測試環境能力決定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="82" customHeight="1">
+      <c r="A6" t="inlineStr" s="13">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="13">
+        <is>
+          <t>TC-LOGIN-001</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="13">
+        <is>
+          <t>SC-LOGIN-001</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="12">
+        <is>
+          <t>有效帳密登入成功</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於登入頁
+2. 測試帳號已存在且密碼正確</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr" s="12">
+        <is>
+          <t>1. 輸入有效帳號
+2. 輸入正確密碼
+3. 送出登入</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統登入成功
+2. 導向登入後首頁或顯示已登入狀態</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr" s="12">
+        <is>
+          <t>成功導向 URL 或畫面狀態需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="82" customHeight="1">
+      <c r="A7" t="inlineStr" s="13">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="13">
+        <is>
+          <t>TC-LOGIN-002</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="13">
+        <is>
+          <t>SC-LOGIN-002</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="12">
+        <is>
+          <t>未輸入帳號時提示必填</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於登入頁</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr" s="12">
+        <is>
+          <t>1. 保留帳號欄位空白
+2. 輸入任意密碼
+3. 送出登入</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統提示帳號為必填
+2. 不應登入成功</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr" s="12">
+        <is>
+          <t>提示文案需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="82" customHeight="1">
+      <c r="A8" t="inlineStr" s="13">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="13">
+        <is>
+          <t>TC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="13">
+        <is>
+          <t>SC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="12">
+        <is>
+          <t>未輸入密碼時提示必填</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於登入頁</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr" s="12">
+        <is>
+          <t>1. 輸入有效帳號
+2. 保留密碼欄位空白
+3. 送出登入</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統提示密碼為必填
+2. 不應登入成功</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr" s="12">
+        <is>
+          <t>提示文案需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="82" customHeight="1">
+      <c r="A9" t="inlineStr" s="13">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="13">
+        <is>
+          <t>TC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="13">
+        <is>
+          <t>SC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="12">
+        <is>
+          <t>錯誤帳密登入失敗</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於登入頁</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr" s="12">
+        <is>
+          <t>1. 輸入錯誤帳號或錯誤密碼
+2. 送出登入</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統顯示登入失敗提示
+2. 不應建立登入狀態</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr" s="12">
+        <is>
+          <t>失敗提示文案待 PM 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="82" customHeight="1">
+      <c r="A10" t="inlineStr" s="13">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="13">
+        <is>
+          <t>TC-LOGIN-005</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="13">
+        <is>
+          <t>SC-LOGIN-005</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="12">
+        <is>
+          <t>忘記密碼入口導向正確</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於登入頁</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr" s="12">
+        <is>
+          <t>1. 點擊忘記密碼入口</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統進入忘記密碼流程</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr" s="12">
+        <is>
+          <t>導向 URL 或頁面標題需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="82" customHeight="1">
+      <c r="A11" t="inlineStr" s="13">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="13">
+        <is>
+          <t>TC-LOGIN-006</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="13">
+        <is>
+          <t>SC-LOGIN-006</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="12">
+        <is>
+          <t>創建帳號入口導向正確</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於登入頁</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr" s="12">
+        <is>
+          <t>1. 點擊創建帳號入口</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統進入註冊流程</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr" s="12">
+        <is>
+          <t>導向 URL 或頁面標題需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="82" customHeight="1">
+      <c r="A12" t="inlineStr" s="13">
+        <is>
+          <t>register</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="13">
+        <is>
+          <t>TC-REGISTER-001</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="13">
+        <is>
+          <t>SC-REGISTER-001</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="12">
+        <is>
+          <t>創建帳號入口導向正確</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於登入頁</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr" s="12">
+        <is>
+          <t>1. 點擊創建帳號入口</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統進入註冊流程</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr" s="12">
+        <is>
+          <t>導向 URL 或頁面狀態需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="82" customHeight="1">
+      <c r="A13" t="inlineStr" s="13">
+        <is>
+          <t>register</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="13">
+        <is>
+          <t>TC-REGISTER-002</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="13">
+        <is>
+          <t>SC-REGISTER-002</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="12">
+        <is>
+          <t>註冊必填欄位未填時提示必填</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於註冊頁</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr" s="12">
+        <is>
+          <t>1. 保留必填欄位空白
+2. 送出註冊</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統提示必填欄位
+2. 不應建立帳號</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr" s="12">
+        <is>
+          <t>必填欄位清單需依 PM Answer 或實作確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="82" customHeight="1">
+      <c r="A14" t="inlineStr" s="13">
+        <is>
+          <t>register</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="13">
+        <is>
+          <t>TC-REGISTER-003</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="13">
+        <is>
+          <t>SC-REGISTER-003</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="12">
+        <is>
+          <t>密碼與確認密碼不一致時提示錯誤</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於註冊頁</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr" s="12">
+        <is>
+          <t>1. 輸入有效基本資料
+2. 輸入不同的密碼與確認密碼
+3. 送出註冊</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統提示密碼不一致
+2. 不應建立帳號</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr" s="12">
+        <is>
+          <t>提示文案需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="82" customHeight="1">
+      <c r="A15" t="inlineStr" s="13">
+        <is>
+          <t>register</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="13">
+        <is>
+          <t>TC-REGISTER-004</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="13">
+        <is>
+          <t>SC-REGISTER-004</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="12">
+        <is>
+          <t>輸入有效資料後建立帳號或進入驗證流程</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr" s="13">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr" s="13">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr" s="12">
+        <is>
+          <t>1. 使用者位於註冊頁
+2. 測試資料未被註冊過</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr" s="12">
+        <is>
+          <t>1. 輸入有效註冊資料
+2. 送出註冊</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr" s="12">
+        <is>
+          <t>1. 系統建立帳號或進入後續驗證流程</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr" s="13">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr" s="12">
+        <is>
+          <t>後續驗證流程與測試資料產生方式需依 PM Answer 確認。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
 </worksheet>
 </file>
</xml_diff>